<commit_message>
Updating the model for Anto
</commit_message>
<xml_diff>
--- a/Anto/Results_Production_Anto_DAM_Corrected_Intraday_15min.xlsx
+++ b/Anto/Results_Production_Anto_DAM_Corrected_Intraday_15min.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="47" uniqueCount="13">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="45" uniqueCount="13">
   <si>
     <t>Data</t>
   </si>
@@ -414,7 +414,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:L36"/>
+  <dimension ref="A1:L34"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:12">
@@ -457,31 +457,31 @@
     </row>
     <row r="2" spans="1:12">
       <c r="A2" s="2">
-        <v>46245.63541666666</v>
+        <v>46253.65625</v>
       </c>
       <c r="B2">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="C2">
-        <v>0.159</v>
+        <v>0.09</v>
       </c>
       <c r="D2">
-        <v>-0.004</v>
+        <v>0.013</v>
       </c>
       <c r="E2">
-        <v>0.155</v>
+        <v>0.103</v>
       </c>
       <c r="F2" s="2">
-        <v>46245.625</v>
+        <v>46253.64583333334</v>
       </c>
       <c r="G2">
-        <v>0.1552938900888889</v>
+        <v>0.1028695888714028</v>
       </c>
       <c r="H2">
-        <v>0.159</v>
+        <v>0.09</v>
       </c>
       <c r="I2">
-        <v>-0.004</v>
+        <v>0.013</v>
       </c>
       <c r="J2">
         <v>1</v>
@@ -495,31 +495,31 @@
     </row>
     <row r="3" spans="1:12">
       <c r="A3" s="2">
-        <v>46245.64583333334</v>
+        <v>46253.66666666666</v>
       </c>
       <c r="B3">
-        <v>63</v>
+        <v>65</v>
       </c>
       <c r="C3">
-        <v>0.136</v>
+        <v>0.08799999999999999</v>
       </c>
       <c r="D3">
-        <v>-0.003</v>
+        <v>0.012</v>
       </c>
       <c r="E3">
-        <v>0.133</v>
+        <v>0.1</v>
       </c>
       <c r="F3" s="2">
-        <v>46245.625</v>
+        <v>46253.64583333334</v>
       </c>
       <c r="G3">
-        <v>0.1552938900888889</v>
+        <v>0.1028695888714028</v>
       </c>
       <c r="H3">
-        <v>0.159</v>
+        <v>0.09</v>
       </c>
       <c r="I3">
-        <v>-0.004</v>
+        <v>0.013</v>
       </c>
       <c r="J3">
         <v>0.917</v>
@@ -533,31 +533,31 @@
     </row>
     <row r="4" spans="1:12">
       <c r="A4" s="2">
-        <v>46245.65625</v>
+        <v>46253.67708333334</v>
       </c>
       <c r="B4">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="C4">
-        <v>0.131</v>
+        <v>0.079</v>
       </c>
       <c r="D4">
-        <v>-0.003</v>
+        <v>0.011</v>
       </c>
       <c r="E4">
-        <v>0.128</v>
+        <v>0.09</v>
       </c>
       <c r="F4" s="2">
-        <v>46245.625</v>
+        <v>46253.64583333334</v>
       </c>
       <c r="G4">
-        <v>0.1552938900888889</v>
+        <v>0.1028695888714028</v>
       </c>
       <c r="H4">
-        <v>0.159</v>
+        <v>0.09</v>
       </c>
       <c r="I4">
-        <v>-0.004</v>
+        <v>0.013</v>
       </c>
       <c r="J4">
         <v>0.8409</v>
@@ -571,31 +571,31 @@
     </row>
     <row r="5" spans="1:12">
       <c r="A5" s="2">
-        <v>46245.66666666666</v>
+        <v>46253.6875</v>
       </c>
       <c r="B5">
-        <v>65</v>
+        <v>67</v>
       </c>
       <c r="C5">
-        <v>0.121</v>
+        <v>0.083</v>
       </c>
       <c r="D5">
-        <v>-0.003</v>
+        <v>0.01</v>
       </c>
       <c r="E5">
-        <v>0.118</v>
+        <v>0.093</v>
       </c>
       <c r="F5" s="2">
-        <v>46245.625</v>
+        <v>46253.64583333334</v>
       </c>
       <c r="G5">
-        <v>0.1552938900888889</v>
+        <v>0.1028695888714028</v>
       </c>
       <c r="H5">
-        <v>0.159</v>
+        <v>0.09</v>
       </c>
       <c r="I5">
-        <v>-0.004</v>
+        <v>0.013</v>
       </c>
       <c r="J5">
         <v>0.7711</v>
@@ -609,31 +609,31 @@
     </row>
     <row r="6" spans="1:12">
       <c r="A6" s="2">
-        <v>46245.67708333334</v>
+        <v>46253.69791666666</v>
       </c>
       <c r="B6">
-        <v>66</v>
+        <v>68</v>
       </c>
       <c r="C6">
-        <v>0.091</v>
+        <v>0.075</v>
       </c>
       <c r="D6">
-        <v>-0.003</v>
+        <v>0.008999999999999999</v>
       </c>
       <c r="E6">
-        <v>0.08799999999999999</v>
+        <v>0.08400000000000001</v>
       </c>
       <c r="F6" s="2">
-        <v>46245.625</v>
+        <v>46253.64583333334</v>
       </c>
       <c r="G6">
-        <v>0.1552938900888889</v>
+        <v>0.1028695888714028</v>
       </c>
       <c r="H6">
-        <v>0.159</v>
+        <v>0.09</v>
       </c>
       <c r="I6">
-        <v>-0.004</v>
+        <v>0.013</v>
       </c>
       <c r="J6">
         <v>0.7071</v>
@@ -647,31 +647,31 @@
     </row>
     <row r="7" spans="1:12">
       <c r="A7" s="2">
-        <v>46245.6875</v>
+        <v>46253.70833333334</v>
       </c>
       <c r="B7">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="C7">
-        <v>0.08500000000000001</v>
+        <v>0.065</v>
       </c>
       <c r="D7">
-        <v>-0.002</v>
+        <v>0.008</v>
       </c>
       <c r="E7">
-        <v>0.083</v>
+        <v>0.073</v>
       </c>
       <c r="F7" s="2">
-        <v>46245.625</v>
+        <v>46253.64583333334</v>
       </c>
       <c r="G7">
-        <v>0.1552938900888889</v>
+        <v>0.1028695888714028</v>
       </c>
       <c r="H7">
-        <v>0.159</v>
+        <v>0.09</v>
       </c>
       <c r="I7">
-        <v>-0.004</v>
+        <v>0.013</v>
       </c>
       <c r="J7">
         <v>0.6484</v>
@@ -685,31 +685,31 @@
     </row>
     <row r="8" spans="1:12">
       <c r="A8" s="2">
-        <v>46245.69791666666</v>
+        <v>46253.71875</v>
       </c>
       <c r="B8">
-        <v>68</v>
+        <v>70</v>
       </c>
       <c r="C8">
-        <v>0.08599999999999999</v>
+        <v>0.06</v>
       </c>
       <c r="D8">
-        <v>-0.002</v>
+        <v>0.008</v>
       </c>
       <c r="E8">
-        <v>0.08400000000000001</v>
+        <v>0.068</v>
       </c>
       <c r="F8" s="2">
-        <v>46245.625</v>
+        <v>46253.64583333334</v>
       </c>
       <c r="G8">
-        <v>0.1552938900888889</v>
+        <v>0.1028695888714028</v>
       </c>
       <c r="H8">
-        <v>0.159</v>
+        <v>0.09</v>
       </c>
       <c r="I8">
-        <v>-0.004</v>
+        <v>0.013</v>
       </c>
       <c r="J8">
         <v>0.5946</v>
@@ -723,31 +723,31 @@
     </row>
     <row r="9" spans="1:12">
       <c r="A9" s="2">
-        <v>46245.70833333334</v>
+        <v>46253.72916666666</v>
       </c>
       <c r="B9">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="C9">
-        <v>0.081</v>
+        <v>0.057</v>
       </c>
       <c r="D9">
-        <v>-0.002</v>
+        <v>0.007</v>
       </c>
       <c r="E9">
-        <v>0.079</v>
+        <v>0.064</v>
       </c>
       <c r="F9" s="2">
-        <v>46245.625</v>
+        <v>46253.64583333334</v>
       </c>
       <c r="G9">
-        <v>0.1552938900888889</v>
+        <v>0.1028695888714028</v>
       </c>
       <c r="H9">
-        <v>0.159</v>
+        <v>0.09</v>
       </c>
       <c r="I9">
-        <v>-0.004</v>
+        <v>0.013</v>
       </c>
       <c r="J9">
         <v>0.5453</v>
@@ -761,31 +761,31 @@
     </row>
     <row r="10" spans="1:12">
       <c r="A10" s="2">
-        <v>46245.71875</v>
+        <v>46253.73958333334</v>
       </c>
       <c r="B10">
-        <v>70</v>
+        <v>72</v>
       </c>
       <c r="C10">
-        <v>0.08500000000000001</v>
+        <v>0.049</v>
       </c>
       <c r="D10">
-        <v>-0.002</v>
+        <v>0.006</v>
       </c>
       <c r="E10">
-        <v>0.083</v>
+        <v>0.055</v>
       </c>
       <c r="F10" s="2">
-        <v>46245.625</v>
+        <v>46253.64583333334</v>
       </c>
       <c r="G10">
-        <v>0.1552938900888889</v>
+        <v>0.1028695888714028</v>
       </c>
       <c r="H10">
-        <v>0.159</v>
+        <v>0.09</v>
       </c>
       <c r="I10">
-        <v>-0.004</v>
+        <v>0.013</v>
       </c>
       <c r="J10">
         <v>0.5</v>
@@ -799,31 +799,31 @@
     </row>
     <row r="11" spans="1:12">
       <c r="A11" s="2">
-        <v>46245.72916666666</v>
+        <v>46253.75</v>
       </c>
       <c r="B11">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="C11">
-        <v>0.078</v>
+        <v>0.044</v>
       </c>
       <c r="D11">
-        <v>-0.002</v>
+        <v>0.006</v>
       </c>
       <c r="E11">
-        <v>0.076</v>
+        <v>0.05</v>
       </c>
       <c r="F11" s="2">
-        <v>46245.625</v>
+        <v>46253.64583333334</v>
       </c>
       <c r="G11">
-        <v>0.1552938900888889</v>
+        <v>0.1028695888714028</v>
       </c>
       <c r="H11">
-        <v>0.159</v>
+        <v>0.09</v>
       </c>
       <c r="I11">
-        <v>-0.004</v>
+        <v>0.013</v>
       </c>
       <c r="J11">
         <v>0.4585</v>
@@ -837,31 +837,31 @@
     </row>
     <row r="12" spans="1:12">
       <c r="A12" s="2">
-        <v>46245.73958333334</v>
+        <v>46253.76041666666</v>
       </c>
       <c r="B12">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="C12">
-        <v>0.067</v>
+        <v>0.041</v>
       </c>
       <c r="D12">
-        <v>-0.002</v>
+        <v>0.005</v>
       </c>
       <c r="E12">
-        <v>0.065</v>
+        <v>0.046</v>
       </c>
       <c r="F12" s="2">
-        <v>46245.625</v>
+        <v>46253.64583333334</v>
       </c>
       <c r="G12">
-        <v>0.1552938900888889</v>
+        <v>0.1028695888714028</v>
       </c>
       <c r="H12">
-        <v>0.159</v>
+        <v>0.09</v>
       </c>
       <c r="I12">
-        <v>-0.004</v>
+        <v>0.013</v>
       </c>
       <c r="J12">
         <v>0.4204</v>
@@ -875,31 +875,31 @@
     </row>
     <row r="13" spans="1:12">
       <c r="A13" s="2">
-        <v>46245.75</v>
+        <v>46253.77083333334</v>
       </c>
       <c r="B13">
-        <v>73</v>
+        <v>75</v>
       </c>
       <c r="C13">
-        <v>0.062</v>
+        <v>0.034</v>
       </c>
       <c r="D13">
-        <v>-0.001</v>
+        <v>0.005</v>
       </c>
       <c r="E13">
-        <v>0.061</v>
+        <v>0.039</v>
       </c>
       <c r="F13" s="2">
-        <v>46245.625</v>
+        <v>46253.64583333334</v>
       </c>
       <c r="G13">
-        <v>0.1552938900888889</v>
+        <v>0.1028695888714028</v>
       </c>
       <c r="H13">
-        <v>0.159</v>
+        <v>0.09</v>
       </c>
       <c r="I13">
-        <v>-0.004</v>
+        <v>0.013</v>
       </c>
       <c r="J13">
         <v>0.3856</v>
@@ -913,31 +913,31 @@
     </row>
     <row r="14" spans="1:12">
       <c r="A14" s="2">
-        <v>46245.76041666666</v>
+        <v>46253.78125</v>
       </c>
       <c r="B14">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="C14">
-        <v>0.055</v>
+        <v>0.027</v>
       </c>
       <c r="D14">
-        <v>-0.001</v>
+        <v>0.005</v>
       </c>
       <c r="E14">
-        <v>0.054</v>
+        <v>0.032</v>
       </c>
       <c r="F14" s="2">
-        <v>46245.625</v>
+        <v>46253.64583333334</v>
       </c>
       <c r="G14">
-        <v>0.1552938900888889</v>
+        <v>0.1028695888714028</v>
       </c>
       <c r="H14">
-        <v>0.159</v>
+        <v>0.09</v>
       </c>
       <c r="I14">
-        <v>-0.004</v>
+        <v>0.013</v>
       </c>
       <c r="J14">
         <v>0.3536</v>
@@ -951,31 +951,31 @@
     </row>
     <row r="15" spans="1:12">
       <c r="A15" s="2">
-        <v>46245.77083333334</v>
+        <v>46253.79166666666</v>
       </c>
       <c r="B15">
-        <v>75</v>
+        <v>77</v>
       </c>
       <c r="C15">
-        <v>0.039</v>
+        <v>0.021</v>
       </c>
       <c r="D15">
-        <v>-0.001</v>
+        <v>0.004</v>
       </c>
       <c r="E15">
-        <v>0.038</v>
+        <v>0.025</v>
       </c>
       <c r="F15" s="2">
-        <v>46245.625</v>
+        <v>46253.64583333334</v>
       </c>
       <c r="G15">
-        <v>0.1552938900888889</v>
+        <v>0.1028695888714028</v>
       </c>
       <c r="H15">
-        <v>0.159</v>
+        <v>0.09</v>
       </c>
       <c r="I15">
-        <v>-0.004</v>
+        <v>0.013</v>
       </c>
       <c r="J15">
         <v>0.3242</v>
@@ -989,31 +989,31 @@
     </row>
     <row r="16" spans="1:12">
       <c r="A16" s="2">
-        <v>46245.78125</v>
+        <v>46253.80208333334</v>
       </c>
       <c r="B16">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="C16">
-        <v>0.033</v>
+        <v>0.016</v>
       </c>
       <c r="D16">
-        <v>-0.001</v>
+        <v>0.004</v>
       </c>
       <c r="E16">
-        <v>0.032</v>
+        <v>0.02</v>
       </c>
       <c r="F16" s="2">
-        <v>46245.625</v>
+        <v>46253.64583333334</v>
       </c>
       <c r="G16">
-        <v>0.1552938900888889</v>
+        <v>0.1028695888714028</v>
       </c>
       <c r="H16">
-        <v>0.159</v>
+        <v>0.09</v>
       </c>
       <c r="I16">
-        <v>-0.004</v>
+        <v>0.013</v>
       </c>
       <c r="J16">
         <v>0.2973</v>
@@ -1027,31 +1027,31 @@
     </row>
     <row r="17" spans="1:12">
       <c r="A17" s="2">
-        <v>46245.79166666666</v>
+        <v>46253.8125</v>
       </c>
       <c r="B17">
-        <v>77</v>
+        <v>79</v>
       </c>
       <c r="C17">
-        <v>0.023</v>
+        <v>0.013</v>
       </c>
       <c r="D17">
-        <v>-0.001</v>
+        <v>0.004</v>
       </c>
       <c r="E17">
-        <v>0.022</v>
+        <v>0.017</v>
       </c>
       <c r="F17" s="2">
-        <v>46245.625</v>
+        <v>46253.64583333334</v>
       </c>
       <c r="G17">
-        <v>0.1552938900888889</v>
+        <v>0.1028695888714028</v>
       </c>
       <c r="H17">
-        <v>0.159</v>
+        <v>0.09</v>
       </c>
       <c r="I17">
-        <v>-0.004</v>
+        <v>0.013</v>
       </c>
       <c r="J17">
         <v>0.2726</v>
@@ -1065,31 +1065,31 @@
     </row>
     <row r="18" spans="1:12">
       <c r="A18" s="2">
-        <v>46245.80208333334</v>
+        <v>46253.82291666666</v>
       </c>
       <c r="B18">
-        <v>78</v>
+        <v>80</v>
       </c>
       <c r="C18">
-        <v>0.02</v>
+        <v>0</v>
       </c>
       <c r="D18">
-        <v>-0.001</v>
+        <v>0.003</v>
       </c>
       <c r="E18">
-        <v>0.019</v>
+        <v>0.003</v>
       </c>
       <c r="F18" s="2">
-        <v>46245.625</v>
+        <v>46253.64583333334</v>
       </c>
       <c r="G18">
-        <v>0.1552938900888889</v>
+        <v>0.1028695888714028</v>
       </c>
       <c r="H18">
-        <v>0.159</v>
+        <v>0.09</v>
       </c>
       <c r="I18">
-        <v>-0.004</v>
+        <v>0.013</v>
       </c>
       <c r="J18">
         <v>0.25</v>
@@ -1103,31 +1103,31 @@
     </row>
     <row r="19" spans="1:12">
       <c r="A19" s="2">
-        <v>46245.8125</v>
+        <v>46253.83333333334</v>
       </c>
       <c r="B19">
-        <v>79</v>
+        <v>81</v>
       </c>
       <c r="C19">
-        <v>0.017</v>
+        <v>0</v>
       </c>
       <c r="D19">
-        <v>-0.001</v>
+        <v>0.003</v>
       </c>
       <c r="E19">
-        <v>0.016</v>
+        <v>0.003</v>
       </c>
       <c r="F19" s="2">
-        <v>46245.625</v>
+        <v>46253.64583333334</v>
       </c>
       <c r="G19">
-        <v>0.1552938900888889</v>
+        <v>0.1028695888714028</v>
       </c>
       <c r="H19">
-        <v>0.159</v>
+        <v>0.09</v>
       </c>
       <c r="I19">
-        <v>-0.004</v>
+        <v>0.013</v>
       </c>
       <c r="J19">
         <v>0.2293</v>
@@ -1141,31 +1141,31 @@
     </row>
     <row r="20" spans="1:12">
       <c r="A20" s="2">
-        <v>46245.82291666666</v>
+        <v>46253.84375</v>
       </c>
       <c r="B20">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="C20">
-        <v>0.011</v>
+        <v>0</v>
       </c>
       <c r="D20">
-        <v>-0.001</v>
+        <v>0.003</v>
       </c>
       <c r="E20">
-        <v>0.01</v>
+        <v>0.003</v>
       </c>
       <c r="F20" s="2">
-        <v>46245.625</v>
+        <v>46253.64583333334</v>
       </c>
       <c r="G20">
-        <v>0.1552938900888889</v>
+        <v>0.1028695888714028</v>
       </c>
       <c r="H20">
-        <v>0.159</v>
+        <v>0.09</v>
       </c>
       <c r="I20">
-        <v>-0.004</v>
+        <v>0.013</v>
       </c>
       <c r="J20">
         <v>0.2102</v>
@@ -1179,31 +1179,31 @@
     </row>
     <row r="21" spans="1:12">
       <c r="A21" s="2">
-        <v>46245.83333333334</v>
+        <v>46253.85416666666</v>
       </c>
       <c r="B21">
-        <v>81</v>
+        <v>83</v>
       </c>
       <c r="C21">
         <v>0</v>
       </c>
       <c r="D21">
-        <v>-0.001</v>
+        <v>0.002</v>
       </c>
       <c r="E21">
-        <v>0</v>
+        <v>0.002</v>
       </c>
       <c r="F21" s="2">
-        <v>46245.625</v>
+        <v>46253.64583333334</v>
       </c>
       <c r="G21">
-        <v>0.1552938900888889</v>
+        <v>0.1028695888714028</v>
       </c>
       <c r="H21">
-        <v>0.159</v>
+        <v>0.09</v>
       </c>
       <c r="I21">
-        <v>-0.004</v>
+        <v>0.013</v>
       </c>
       <c r="J21">
         <v>0.1928</v>
@@ -1217,31 +1217,31 @@
     </row>
     <row r="22" spans="1:12">
       <c r="A22" s="2">
-        <v>46245.84375</v>
+        <v>46253.86458333334</v>
       </c>
       <c r="B22">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="C22">
         <v>0</v>
       </c>
       <c r="D22">
-        <v>-0.001</v>
+        <v>-0</v>
       </c>
       <c r="E22">
         <v>0</v>
       </c>
       <c r="F22" s="2">
-        <v>46245.625</v>
+        <v>46253.64583333334</v>
       </c>
       <c r="G22">
-        <v>0.1552938900888889</v>
+        <v>0.1028695888714028</v>
       </c>
       <c r="H22">
-        <v>0.159</v>
+        <v>0.09</v>
       </c>
       <c r="I22">
-        <v>-0.004</v>
+        <v>0.013</v>
       </c>
       <c r="J22">
         <v>0.1768</v>
@@ -1255,31 +1255,31 @@
     </row>
     <row r="23" spans="1:12">
       <c r="A23" s="2">
-        <v>46245.85416666666</v>
+        <v>46253.875</v>
       </c>
       <c r="B23">
-        <v>83</v>
+        <v>85</v>
       </c>
       <c r="C23">
         <v>0</v>
       </c>
       <c r="D23">
-        <v>-0.001</v>
+        <v>-0</v>
       </c>
       <c r="E23">
         <v>0</v>
       </c>
       <c r="F23" s="2">
-        <v>46245.625</v>
+        <v>46253.64583333334</v>
       </c>
       <c r="G23">
-        <v>0.1552938900888889</v>
+        <v>0.1028695888714028</v>
       </c>
       <c r="H23">
-        <v>0.159</v>
+        <v>0.09</v>
       </c>
       <c r="I23">
-        <v>-0.004</v>
+        <v>0.013</v>
       </c>
       <c r="J23">
         <v>0.1621</v>
@@ -1293,31 +1293,31 @@
     </row>
     <row r="24" spans="1:12">
       <c r="A24" s="2">
-        <v>46245.86458333334</v>
+        <v>46253.88541666666</v>
       </c>
       <c r="B24">
-        <v>84</v>
+        <v>86</v>
       </c>
       <c r="C24">
         <v>0</v>
       </c>
       <c r="D24">
-        <v>-0.001</v>
+        <v>-0</v>
       </c>
       <c r="E24">
         <v>0</v>
       </c>
       <c r="F24" s="2">
-        <v>46245.625</v>
+        <v>46253.64583333334</v>
       </c>
       <c r="G24">
-        <v>0.1552938900888889</v>
+        <v>0.1028695888714028</v>
       </c>
       <c r="H24">
-        <v>0.159</v>
+        <v>0.09</v>
       </c>
       <c r="I24">
-        <v>-0.004</v>
+        <v>0.013</v>
       </c>
       <c r="J24">
         <v>0.1487</v>
@@ -1331,10 +1331,10 @@
     </row>
     <row r="25" spans="1:12">
       <c r="A25" s="2">
-        <v>46245.875</v>
+        <v>46253.89583333334</v>
       </c>
       <c r="B25">
-        <v>85</v>
+        <v>87</v>
       </c>
       <c r="C25">
         <v>0</v>
@@ -1346,16 +1346,16 @@
         <v>0</v>
       </c>
       <c r="F25" s="2">
-        <v>46245.625</v>
+        <v>46253.64583333334</v>
       </c>
       <c r="G25">
-        <v>0.1552938900888889</v>
+        <v>0.1028695888714028</v>
       </c>
       <c r="H25">
-        <v>0.159</v>
+        <v>0.09</v>
       </c>
       <c r="I25">
-        <v>-0.004</v>
+        <v>0.013</v>
       </c>
       <c r="J25">
         <v>0.1363</v>
@@ -1369,10 +1369,10 @@
     </row>
     <row r="26" spans="1:12">
       <c r="A26" s="2">
-        <v>46245.88541666666</v>
+        <v>46253.90625</v>
       </c>
       <c r="B26">
-        <v>86</v>
+        <v>88</v>
       </c>
       <c r="C26">
         <v>0</v>
@@ -1384,16 +1384,16 @@
         <v>0</v>
       </c>
       <c r="F26" s="2">
-        <v>46245.625</v>
+        <v>46253.64583333334</v>
       </c>
       <c r="G26">
-        <v>0.1552938900888889</v>
+        <v>0.1028695888714028</v>
       </c>
       <c r="H26">
-        <v>0.159</v>
+        <v>0.09</v>
       </c>
       <c r="I26">
-        <v>-0.004</v>
+        <v>0.013</v>
       </c>
       <c r="J26">
         <v>0.125</v>
@@ -1407,10 +1407,10 @@
     </row>
     <row r="27" spans="1:12">
       <c r="A27" s="2">
-        <v>46245.89583333334</v>
+        <v>46253.91666666666</v>
       </c>
       <c r="B27">
-        <v>87</v>
+        <v>89</v>
       </c>
       <c r="C27">
         <v>0</v>
@@ -1422,16 +1422,16 @@
         <v>0</v>
       </c>
       <c r="F27" s="2">
-        <v>46245.625</v>
+        <v>46253.64583333334</v>
       </c>
       <c r="G27">
-        <v>0.1552938900888889</v>
+        <v>0.1028695888714028</v>
       </c>
       <c r="H27">
-        <v>0.159</v>
+        <v>0.09</v>
       </c>
       <c r="I27">
-        <v>-0.004</v>
+        <v>0.013</v>
       </c>
       <c r="J27">
         <v>0.1146</v>
@@ -1445,10 +1445,10 @@
     </row>
     <row r="28" spans="1:12">
       <c r="A28" s="2">
-        <v>46245.90625</v>
+        <v>46253.92708333334</v>
       </c>
       <c r="B28">
-        <v>88</v>
+        <v>90</v>
       </c>
       <c r="C28">
         <v>0</v>
@@ -1460,16 +1460,16 @@
         <v>0</v>
       </c>
       <c r="F28" s="2">
-        <v>46245.625</v>
+        <v>46253.64583333334</v>
       </c>
       <c r="G28">
-        <v>0.1552938900888889</v>
+        <v>0.1028695888714028</v>
       </c>
       <c r="H28">
-        <v>0.159</v>
+        <v>0.09</v>
       </c>
       <c r="I28">
-        <v>-0.004</v>
+        <v>0.013</v>
       </c>
       <c r="J28">
         <v>0.1051</v>
@@ -1483,10 +1483,10 @@
     </row>
     <row r="29" spans="1:12">
       <c r="A29" s="2">
-        <v>46245.91666666666</v>
+        <v>46253.9375</v>
       </c>
       <c r="B29">
-        <v>89</v>
+        <v>91</v>
       </c>
       <c r="C29">
         <v>0</v>
@@ -1498,16 +1498,16 @@
         <v>0</v>
       </c>
       <c r="F29" s="2">
-        <v>46245.625</v>
+        <v>46253.64583333334</v>
       </c>
       <c r="G29">
-        <v>0.1552938900888889</v>
+        <v>0.1028695888714028</v>
       </c>
       <c r="H29">
-        <v>0.159</v>
+        <v>0.09</v>
       </c>
       <c r="I29">
-        <v>-0.004</v>
+        <v>0.013</v>
       </c>
       <c r="J29">
         <v>0.0964</v>
@@ -1521,10 +1521,10 @@
     </row>
     <row r="30" spans="1:12">
       <c r="A30" s="2">
-        <v>46245.92708333334</v>
+        <v>46253.94791666666</v>
       </c>
       <c r="B30">
-        <v>90</v>
+        <v>92</v>
       </c>
       <c r="C30">
         <v>0</v>
@@ -1536,16 +1536,16 @@
         <v>0</v>
       </c>
       <c r="F30" s="2">
-        <v>46245.625</v>
+        <v>46253.64583333334</v>
       </c>
       <c r="G30">
-        <v>0.1552938900888889</v>
+        <v>0.1028695888714028</v>
       </c>
       <c r="H30">
-        <v>0.159</v>
+        <v>0.09</v>
       </c>
       <c r="I30">
-        <v>-0.004</v>
+        <v>0.013</v>
       </c>
       <c r="J30">
         <v>0.08840000000000001</v>
@@ -1559,10 +1559,10 @@
     </row>
     <row r="31" spans="1:12">
       <c r="A31" s="2">
-        <v>46245.9375</v>
+        <v>46253.95833333334</v>
       </c>
       <c r="B31">
-        <v>91</v>
+        <v>93</v>
       </c>
       <c r="C31">
         <v>0</v>
@@ -1574,16 +1574,16 @@
         <v>0</v>
       </c>
       <c r="F31" s="2">
-        <v>46245.625</v>
+        <v>46253.64583333334</v>
       </c>
       <c r="G31">
-        <v>0.1552938900888889</v>
+        <v>0.1028695888714028</v>
       </c>
       <c r="H31">
-        <v>0.159</v>
+        <v>0.09</v>
       </c>
       <c r="I31">
-        <v>-0.004</v>
+        <v>0.013</v>
       </c>
       <c r="J31">
         <v>0.08110000000000001</v>
@@ -1597,10 +1597,10 @@
     </row>
     <row r="32" spans="1:12">
       <c r="A32" s="2">
-        <v>46245.94791666666</v>
+        <v>46253.96875</v>
       </c>
       <c r="B32">
-        <v>92</v>
+        <v>94</v>
       </c>
       <c r="C32">
         <v>0</v>
@@ -1612,16 +1612,16 @@
         <v>0</v>
       </c>
       <c r="F32" s="2">
-        <v>46245.625</v>
+        <v>46253.64583333334</v>
       </c>
       <c r="G32">
-        <v>0.1552938900888889</v>
+        <v>0.1028695888714028</v>
       </c>
       <c r="H32">
-        <v>0.159</v>
+        <v>0.09</v>
       </c>
       <c r="I32">
-        <v>-0.004</v>
+        <v>0.013</v>
       </c>
       <c r="J32">
         <v>0.0743</v>
@@ -1635,10 +1635,10 @@
     </row>
     <row r="33" spans="1:12">
       <c r="A33" s="2">
-        <v>46245.95833333334</v>
+        <v>46253.97916666666</v>
       </c>
       <c r="B33">
-        <v>93</v>
+        <v>95</v>
       </c>
       <c r="C33">
         <v>0</v>
@@ -1650,16 +1650,16 @@
         <v>0</v>
       </c>
       <c r="F33" s="2">
-        <v>46245.625</v>
+        <v>46253.64583333334</v>
       </c>
       <c r="G33">
-        <v>0.1552938900888889</v>
+        <v>0.1028695888714028</v>
       </c>
       <c r="H33">
-        <v>0.159</v>
+        <v>0.09</v>
       </c>
       <c r="I33">
-        <v>-0.004</v>
+        <v>0.013</v>
       </c>
       <c r="J33">
         <v>0.0682</v>
@@ -1673,10 +1673,10 @@
     </row>
     <row r="34" spans="1:12">
       <c r="A34" s="2">
-        <v>46245.96875</v>
+        <v>46253.98958333334</v>
       </c>
       <c r="B34">
-        <v>94</v>
+        <v>96</v>
       </c>
       <c r="C34">
         <v>0</v>
@@ -1688,16 +1688,16 @@
         <v>0</v>
       </c>
       <c r="F34" s="2">
-        <v>46245.625</v>
+        <v>46253.64583333334</v>
       </c>
       <c r="G34">
-        <v>0.1552938900888889</v>
+        <v>0.1028695888714028</v>
       </c>
       <c r="H34">
-        <v>0.159</v>
+        <v>0.09</v>
       </c>
       <c r="I34">
-        <v>-0.004</v>
+        <v>0.013</v>
       </c>
       <c r="J34">
         <v>0.0625</v>
@@ -1706,82 +1706,6 @@
         <v>495</v>
       </c>
       <c r="L34" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="35" spans="1:12">
-      <c r="A35" s="2">
-        <v>46245.97916666666</v>
-      </c>
-      <c r="B35">
-        <v>95</v>
-      </c>
-      <c r="C35">
-        <v>0</v>
-      </c>
-      <c r="D35">
-        <v>-0</v>
-      </c>
-      <c r="E35">
-        <v>0</v>
-      </c>
-      <c r="F35" s="2">
-        <v>46245.625</v>
-      </c>
-      <c r="G35">
-        <v>0.1552938900888889</v>
-      </c>
-      <c r="H35">
-        <v>0.159</v>
-      </c>
-      <c r="I35">
-        <v>-0.004</v>
-      </c>
-      <c r="J35">
-        <v>0.0573</v>
-      </c>
-      <c r="K35">
-        <v>510</v>
-      </c>
-      <c r="L35" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="36" spans="1:12">
-      <c r="A36" s="2">
-        <v>46245.98958333334</v>
-      </c>
-      <c r="B36">
-        <v>96</v>
-      </c>
-      <c r="C36">
-        <v>0</v>
-      </c>
-      <c r="D36">
-        <v>-0</v>
-      </c>
-      <c r="E36">
-        <v>0</v>
-      </c>
-      <c r="F36" s="2">
-        <v>46245.625</v>
-      </c>
-      <c r="G36">
-        <v>0.1552938900888889</v>
-      </c>
-      <c r="H36">
-        <v>0.159</v>
-      </c>
-      <c r="I36">
-        <v>-0.004</v>
-      </c>
-      <c r="J36">
-        <v>0.0526</v>
-      </c>
-      <c r="K36">
-        <v>525</v>
-      </c>
-      <c r="L36" t="s">
         <v>12</v>
       </c>
     </row>

</xml_diff>